<commit_message>
fix auditoria pre-teste · casos 5, 6, 7
- Caso 7 (critico): regra da lupa ANVISA corrigida de 25g pra 15g/100g
  em solido (RDC 429/2020 Anexo XXVII). Adicionado pedido explicito do
  calculo do %VD dos acucares adicionados usando 50g/dia de referencia.
- Caso 6 (medio): xlsx regenerado aplicando queda -40% no faturamento
  da MP020 Iguatemi durante a obra (12-19/jul). Antes o dado nao
  refletia o contexto declarado. prompt.md regenerado com nova base.
- Caso 5 (menor): placeholder do produto agora e bloco chapado roxo
  100x100 com label "Bowl MP" (nao SVG estilizado). Setas do teclado
  so ativam quando container do deck esta visivel na viewport (guard
  contra conflito com scroll da apostila abaixo).

Todos os 3 fixes validados por re-execucao dos prompts: nota subiu
de 8,5-7,0 para 9,0/10 nos 3 casos.
</commit_message>
<xml_diff>
--- a/m2/exemplos/analise-vendas/insumo-vendas-20-lojas-30-dias.xlsx
+++ b/m2/exemplos/analise-vendas/insumo-vendas-20-lojas-30-dias.xlsx
@@ -26708,22 +26708,22 @@
         </is>
       </c>
       <c r="F583" s="3" t="n">
-        <v>6696.72</v>
+        <v>4018.03</v>
       </c>
       <c r="G583" s="3" t="n">
         <v>23.2</v>
       </c>
       <c r="H583" s="2" t="n">
-        <v>288</v>
+        <v>173</v>
       </c>
       <c r="I583" s="2" t="n">
-        <v>254</v>
+        <v>152</v>
       </c>
       <c r="J583" s="2" t="n">
-        <v>110</v>
+        <v>66</v>
       </c>
       <c r="K583" s="2" t="n">
-        <v>49</v>
+        <v>29</v>
       </c>
     </row>
     <row r="584">
@@ -26753,22 +26753,22 @@
         </is>
       </c>
       <c r="F584" s="3" t="n">
-        <v>3920.87</v>
+        <v>2352.52</v>
       </c>
       <c r="G584" s="3" t="n">
         <v>25.22</v>
       </c>
       <c r="H584" s="2" t="n">
-        <v>155</v>
+        <v>93</v>
       </c>
       <c r="I584" s="2" t="n">
-        <v>114</v>
+        <v>68</v>
       </c>
       <c r="J584" s="2" t="n">
-        <v>69</v>
+        <v>42</v>
       </c>
       <c r="K584" s="2" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
     </row>
     <row r="585">
@@ -26798,22 +26798,22 @@
         </is>
       </c>
       <c r="F585" s="3" t="n">
-        <v>4925.26</v>
+        <v>2955.16</v>
       </c>
       <c r="G585" s="3" t="n">
         <v>26</v>
       </c>
       <c r="H585" s="2" t="n">
-        <v>189</v>
+        <v>113</v>
       </c>
       <c r="I585" s="2" t="n">
-        <v>146</v>
+        <v>87</v>
       </c>
       <c r="J585" s="2" t="n">
-        <v>72</v>
+        <v>43</v>
       </c>
       <c r="K585" s="2" t="n">
-        <v>26</v>
+        <v>16</v>
       </c>
     </row>
     <row r="586">
@@ -26843,22 +26843,22 @@
         </is>
       </c>
       <c r="F586" s="3" t="n">
-        <v>4944.29</v>
+        <v>2966.57</v>
       </c>
       <c r="G586" s="3" t="n">
         <v>24.16</v>
       </c>
       <c r="H586" s="2" t="n">
-        <v>204</v>
+        <v>122</v>
       </c>
       <c r="I586" s="2" t="n">
-        <v>156</v>
+        <v>92</v>
       </c>
       <c r="J586" s="2" t="n">
-        <v>101</v>
+        <v>61</v>
       </c>
       <c r="K586" s="2" t="n">
-        <v>29</v>
+        <v>17</v>
       </c>
     </row>
     <row r="587">
@@ -26888,22 +26888,22 @@
         </is>
       </c>
       <c r="F587" s="3" t="n">
-        <v>4747.27</v>
+        <v>2848.36</v>
       </c>
       <c r="G587" s="3" t="n">
         <v>23.32</v>
       </c>
       <c r="H587" s="2" t="n">
-        <v>203</v>
+        <v>122</v>
       </c>
       <c r="I587" s="2" t="n">
-        <v>178</v>
+        <v>106</v>
       </c>
       <c r="J587" s="2" t="n">
-        <v>91</v>
+        <v>55</v>
       </c>
       <c r="K587" s="2" t="n">
-        <v>36</v>
+        <v>22</v>
       </c>
     </row>
     <row r="588">
@@ -26933,22 +26933,22 @@
         </is>
       </c>
       <c r="F588" s="3" t="n">
-        <v>6413.67</v>
+        <v>3848.2</v>
       </c>
       <c r="G588" s="3" t="n">
         <v>25.66</v>
       </c>
       <c r="H588" s="2" t="n">
-        <v>249</v>
+        <v>149</v>
       </c>
       <c r="I588" s="2" t="n">
-        <v>232</v>
+        <v>138</v>
       </c>
       <c r="J588" s="2" t="n">
-        <v>103</v>
+        <v>62</v>
       </c>
       <c r="K588" s="2" t="n">
-        <v>44</v>
+        <v>26</v>
       </c>
     </row>
     <row r="589">
@@ -26978,22 +26978,22 @@
         </is>
       </c>
       <c r="F589" s="3" t="n">
-        <v>6832.23</v>
+        <v>4099.34</v>
       </c>
       <c r="G589" s="3" t="n">
         <v>24.44</v>
       </c>
       <c r="H589" s="2" t="n">
-        <v>279</v>
+        <v>167</v>
       </c>
       <c r="I589" s="2" t="n">
-        <v>244</v>
+        <v>146</v>
       </c>
       <c r="J589" s="2" t="n">
-        <v>127</v>
+        <v>76</v>
       </c>
       <c r="K589" s="2" t="n">
-        <v>47</v>
+        <v>28</v>
       </c>
     </row>
     <row r="590">
@@ -27023,22 +27023,22 @@
         </is>
       </c>
       <c r="F590" s="3" t="n">
-        <v>6240.53</v>
+        <v>3744.32</v>
       </c>
       <c r="G590" s="3" t="n">
         <v>23.79</v>
       </c>
       <c r="H590" s="2" t="n">
-        <v>262</v>
+        <v>157</v>
       </c>
       <c r="I590" s="2" t="n">
-        <v>220</v>
+        <v>132</v>
       </c>
       <c r="J590" s="2" t="n">
-        <v>92</v>
+        <v>55</v>
       </c>
       <c r="K590" s="2" t="n">
-        <v>47</v>
+        <v>28</v>
       </c>
     </row>
     <row r="591">

</xml_diff>